<commit_message>
V2 architecture: DAC ZOH, 8sps channel, dual BER, docs
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,17 +444,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sps_sim</t>
+          <t>sps_dsp</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sps_dsp</t>
+          <t>sps_dac</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -464,10 +464,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>sps_channel</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sps_adc</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>num_symbols</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B7" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -548,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,40 +596,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pd_bw</t>
+          <t>fiber_length_km</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40000000000</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tia_bw</t>
+          <t>fiber_loss_db_km</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35000000000</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>adc_bw</t>
+          <t>pd_bw</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>tia_bw</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>35000000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>adc_bw</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>35000000000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>snr_db</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B8" t="n">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add PCB host trace loss model (CEI-112G standard)
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,57 +586,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mzm_bw</t>
+          <t>pcb_loss_nyquist_db</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35000000000</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fiber_length_km</t>
+          <t>mzm_bw</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>35000000000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fiber_loss_db_km</t>
+          <t>fiber_length_km</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pd_bw</t>
+          <t>fiber_loss_db_km</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40000000000</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tia_bw</t>
+          <t>pd_bw</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>adc_bw</t>
+          <t>tia_bw</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -646,10 +646,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>adc_bw</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>35000000000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>snr_db</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feat: upgrade simulation framework to 448G PAM4/PAM6 with realistic S-parameter channel modeling, IEEE COM CTLE, and LS-initialized FFE
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -438,7 +438,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>56000000000</v>
+        <v>212500000000</v>
       </c>
     </row>
     <row r="3">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,71 +596,143 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mzm_bw</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>35000000000</v>
+          <t>use_s4p</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fiber_length_km</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+          <t>s4p_file</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>models/li_dj_CR_DesignA_060523/li_dj_CR_Design_A_Rev1_THRU.s4p</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fiber_loss_db_km</t>
+          <t>mzm_bw</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4</v>
+        <v>110000000000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pd_bw</t>
+          <t>fiber_length_km</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40000000000</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tia_bw</t>
+          <t>fiber_loss_db_km</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>35000000000</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>adc_bw</t>
+          <t>pd_bw</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35000000000</v>
+        <v>110000000000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>tia_bw</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>110000000000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>adc_bw</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>110000000000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>snr_db</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B11" t="n">
         <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>use_ctle</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ctle_g_dc_db</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ctle_fz_ratio</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ctle_fp1_ratio</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ctle_fp2_ratio</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -696,7 +768,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -706,7 +778,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Fix bugs, apply ZTE init taps, disable DFE, add unified eye plot switch and 50 Sps upsampling
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -438,7 +438,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>212500000000</v>
+        <v>112500000000</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -618,120 +618,140 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mzm_bw</t>
+          <t>s4p_f_scale</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>110000000000</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fiber_length_km</t>
+          <t>target_il_nyquist_db</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fiber_loss_db_km</t>
+          <t>mzm_bw</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4</v>
+        <v>150000000000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pd_bw</t>
+          <t>fiber_length_km</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>110000000000</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tia_bw</t>
+          <t>fiber_loss_db_km</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>110000000000</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>adc_bw</t>
+          <t>pd_bw</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>110000000000</v>
+        <v>150000000000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>snr_db</t>
+          <t>tia_bw</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25</v>
+        <v>150000000000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>use_ctle</t>
-        </is>
-      </c>
-      <c r="B12" t="b">
-        <v>1</v>
+          <t>adc_bw</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>150000000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ctle_g_dc_db</t>
+          <t>snr_db</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ctle_fz_ratio</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2.5</v>
+          <t>use_ctle</t>
+        </is>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ctle_fp1_ratio</t>
+          <t>ctle_g_dc_db</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.5</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>ctle_fz_ratio</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ctle_fp1_ratio</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>ctle_fp2_ratio</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -746,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -784,30 +804,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>lms_mu</t>
+          <t>dfe_taps</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>train_len</t>
+          <t>lms_mu</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2000</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>train_len</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>mlse_memory</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B7" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: support 112G/224G/448G multi-mode, clear old baseline results, update documentation
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,10 +484,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>plot_intermediate_eyes</t>
+        </is>
+      </c>
+      <c r="B7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>num_symbols</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -502,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,17 +530,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ctle_dc_gain</t>
+          <t>baud_rate</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8</v>
+        <v>112500000000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ctle_peaking</t>
+          <t>sps_dac</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -540,22 +550,50 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ffe_taps</t>
+          <t>levels</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ffe_pre</t>
+          <t>pattern_length</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
-      </c>
+        <v>65536</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ffe_taps</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ffe_spacing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>custom_taps</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -586,53 +624,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>pcb_loss_nyquist_db</t>
+          <t>sps_channel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>use_s4p</t>
-        </is>
-      </c>
-      <c r="B3" t="b">
-        <v>1</v>
+          <t>snr_db</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>s4p_file</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>models/li_dj_CR_DesignA_060523/li_dj_CR_Design_A_Rev1_THRU.s4p</t>
-        </is>
+          <t>use_s4p</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>s4p_f_scale</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1.4</v>
+          <t>s4p_file</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>models/li_dj_CR_DesignA_060523/li_dj_CR_Design_A_Rev1_THRU.s4p</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>target_il_nyquist_db</t>
+          <t>s4p_f_scale</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -642,7 +680,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>150000000000</v>
+        <v>80000000000</v>
       </c>
     </row>
     <row r="8">
@@ -662,7 +700,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10">
@@ -672,7 +710,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>150000000000</v>
+        <v>80000000000</v>
       </c>
     </row>
     <row r="11">
@@ -682,7 +720,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>150000000000</v>
+        <v>80000000000</v>
       </c>
     </row>
     <row r="12">
@@ -692,67 +730,67 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>150000000000</v>
+        <v>80000000000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>snr_db</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>25</v>
+          <t>use_ctle</t>
+        </is>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>use_ctle</t>
-        </is>
-      </c>
-      <c r="B14" t="b">
-        <v>1</v>
+          <t>ctle_fz_ratio</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ctle_g_dc_db</t>
+          <t>ctle_fp1_ratio</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-12</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ctle_fz_ratio</t>
+          <t>ctle_fp2_ratio</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ctle_fp1_ratio</t>
+          <t>ctle_g_dc_db</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.5</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ctle_fp2_ratio</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
+          <t>disable_isi</t>
+        </is>
+      </c>
+      <c r="B18" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -766,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -784,61 +822,91 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ffe_taps</t>
+          <t>sps_adc</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ffe_pre</t>
+          <t>ffe_taps</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dfe_taps</t>
+          <t>ffe_spacing</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>lms_mu</t>
+          <t>ffe_pre</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.001</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>train_len</t>
+          <t>ffe_mu</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2000</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>lms_mu</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>train_len</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dfe_taps</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>mlse_memory</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>1</v>
+      <c r="B10" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Integrate ZF FFE + Burg MLSE architecture, disable DFE, and set BO optimal defaults
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -438,7 +438,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112500000000</v>
+        <v>56000000000</v>
       </c>
     </row>
     <row r="3">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
     </row>
   </sheetData>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112500000000</v>
+        <v>56000000000</v>
       </c>
     </row>
     <row r="3">
@@ -593,7 +593,11 @@
           <t>custom_taps</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, -0.2987, 0.7012, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -659,7 +663,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>models/li_dj_CR_DesignA_060523/li_dj_CR_Design_A_Rev1_THRU.s4p</t>
+          <t>models/lim_3ck_01_0319_c2m/lim/100G_C2M_channel_update_part1/Channel1/112G_16dB_(QSFPDD+module card)_TX7_L10/112G_cascaded_CDR6_Module_Thru_1_etch1100_TX7_L10_Full_Footprint.s4p</t>
         </is>
       </c>
     </row>
@@ -680,7 +684,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>80000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="8">
@@ -710,7 +714,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>80000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="11">
@@ -720,7 +724,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="12">
@@ -730,7 +734,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>80000000000</v>
+        <v>40000000000</v>
       </c>
     </row>
     <row r="13">
@@ -780,7 +784,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -886,7 +890,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="9">
@@ -906,7 +910,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add 4-algorithm benchmark and update config for SHC
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>50000</v>
+        <v>2000000</v>
       </c>
     </row>
   </sheetData>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,6 +596,18 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>[0.0, 0.0, 0.0, -0.2987, 0.7012, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>optimizer_type</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SHC</t>
         </is>
       </c>
     </row>
@@ -642,7 +654,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Refactor optimization objective to MLSE BER and validate algorithms
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2000000</v>
+        <v>65536</v>
       </c>
     </row>
   </sheetData>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27.5</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Results: Inject optimal GA 12-param coefficients into config and regenerate diagnostics
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,20 +484,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>plot_intermediate_eyes</t>
+          <t>enable_eye_plot</t>
         </is>
       </c>
       <c r="B7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>enable_spectrum_plot</t>
+        </is>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>num_symbols</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>65536</v>
       </c>
     </row>
@@ -512,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,6 +619,68 @@
         <is>
           <t>SHC</t>
         </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>optimize_mode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>JOINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>use_ctle</t>
+        </is>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ctle_fz_ratio</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ctle_fp1_ratio</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ctle_fp2_ratio</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ctle_g_dc_db</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -622,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -752,60 +824,10 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>use_ctle</t>
+          <t>disable_isi</t>
         </is>
       </c>
       <c r="B13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>ctle_fz_ratio</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>ctle_fp1_ratio</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>ctle_fp2_ratio</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ctle_g_dc_db</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>disable_isi</t>
-        </is>
-      </c>
-      <c r="B18" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implement Safe-BO with soft penalty barrier and add configuration
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -636,27 +636,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>use_ctle</t>
-        </is>
-      </c>
-      <c r="B11" t="b">
-        <v>1</v>
+          <t>safe_bo_max_log_ber</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ctle_fz_ratio</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2.5</v>
+          <t>use_ctle</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ctle_fp1_ratio</t>
+          <t>ctle_fz_ratio</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -666,20 +666,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ctle_fp2_ratio</t>
+          <t>ctle_fp1_ratio</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>ctle_fp2_ratio</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>ctle_g_dc_db</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B16" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(lpo): upgrade channel model and params to LPO MSA standard
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="60">
   <si>
     <t>Parameter</t>
   </si>
@@ -105,6 +105,27 @@
   </si>
   <si>
     <t>snr_db</t>
+  </si>
+  <si>
+    <t>tx_pcb_loss_nyquist_db</t>
+  </si>
+  <si>
+    <t>rx_pcb_loss_nyquist_db</t>
+  </si>
+  <si>
+    <t>use_distributed_noise</t>
+  </si>
+  <si>
+    <t>host_tx_noise_rms</t>
+  </si>
+  <si>
+    <t>module_tx_noise_rms</t>
+  </si>
+  <si>
+    <t>module_rx_noise_rms</t>
+  </si>
+  <si>
+    <t>host_rx_noise_rms</t>
   </si>
   <si>
     <t>use_s4p</t>
@@ -736,7 +757,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -767,23 +788,23 @@
       <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="b">
-        <v>1</v>
+      <c r="B4">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
-        <v>39</v>
+      <c r="B5">
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -792,7 +813,7 @@
         <v>32</v>
       </c>
       <c r="B7">
-        <v>40000000000</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -800,7 +821,7 @@
         <v>33</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -808,7 +829,7 @@
         <v>34</v>
       </c>
       <c r="B9">
-        <v>0.25</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -816,30 +837,86 @@
         <v>35</v>
       </c>
       <c r="B10">
-        <v>40000000000</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="B11">
-        <v>40000000000</v>
+      <c r="B11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>37</v>
       </c>
-      <c r="B12">
-        <v>40000000000</v>
+      <c r="B12" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>38</v>
       </c>
-      <c r="B13" t="b">
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -874,7 +951,7 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -882,20 +959,20 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B6">
         <v>0.0001</v>
@@ -903,7 +980,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B7">
         <v>0.0001</v>
@@ -911,7 +988,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B8">
         <v>10000</v>
@@ -919,18 +996,18 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -945,16 +1022,16 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
         <v>28</v>
@@ -979,7 +1056,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -996,7 +1073,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1013,7 +1090,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B5">
         <v>28</v>

</xml_diff>

<commit_message>
Save progress before SJTU channel modeling
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t>Parameter</t>
   </si>
@@ -92,7 +92,13 @@
     <t>ctle_fp2_ratio</t>
   </si>
   <si>
+    <t>ctle_flf_ratio</t>
+  </si>
+  <si>
     <t>ctle_g_dc_db</t>
+  </si>
+  <si>
+    <t>ctle_g_dc2_db</t>
   </si>
   <si>
     <t>[0.0, 0.0, 0.0, -0.2987, 0.7012, 0.0, 0.0, 0.0, 0.0]</t>
@@ -619,7 +625,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -683,7 +689,7 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -691,7 +697,7 @@
         <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -699,7 +705,7 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -747,6 +753,22 @@
         <v>24</v>
       </c>
       <c r="B16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18">
         <v>0</v>
       </c>
     </row>
@@ -778,7 +800,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>26.5</v>
@@ -786,7 +808,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>7</v>
@@ -794,7 +816,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5">
         <v>7</v>
@@ -802,7 +824,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" t="b">
         <v>1</v>
@@ -810,7 +832,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B7">
         <v>0.003</v>
@@ -818,7 +840,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8">
         <v>0.003</v>
@@ -826,7 +848,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B9">
         <v>0.003</v>
@@ -834,7 +856,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B10">
         <v>0.003</v>
@@ -842,7 +864,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>
@@ -850,15 +872,15 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -866,7 +888,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14">
         <v>40000000000</v>
@@ -874,7 +896,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -882,7 +904,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B16">
         <v>0.25</v>
@@ -890,7 +912,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B17">
         <v>40000000000</v>
@@ -898,7 +920,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B18">
         <v>40000000000</v>
@@ -906,7 +928,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B19">
         <v>40000000000</v>
@@ -914,7 +936,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B20" t="b">
         <v>0</v>
@@ -964,7 +986,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -972,7 +994,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6">
         <v>0.0001</v>
@@ -980,7 +1002,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7">
         <v>0.0001</v>
@@ -988,7 +1010,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8">
         <v>10000</v>
@@ -996,7 +1018,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1004,7 +1026,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1022,19 +1044,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1056,7 +1078,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1073,7 +1095,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -1090,7 +1112,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B5">
         <v>28</v>

</xml_diff>

<commit_message>
Refactor channel noise to physical parameters, remove global SNR, update docs, clean up old datasets and scripts
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
   <si>
     <t>Parameter</t>
   </si>
@@ -110,30 +110,51 @@
     <t>JOINT</t>
   </si>
   <si>
-    <t>snr_db</t>
-  </si>
-  <si>
     <t>tx_pcb_loss_nyquist_db</t>
   </si>
   <si>
     <t>rx_pcb_loss_nyquist_db</t>
   </si>
   <si>
-    <t>use_distributed_noise</t>
+    <t>driver_vpp</t>
+  </si>
+  <si>
+    <t>laser_rin_db_hz</t>
+  </si>
+  <si>
+    <t>mzm_v_pi</t>
+  </si>
+  <si>
+    <t>mzm_v_bias</t>
+  </si>
+  <si>
+    <t>mzm_er_db</t>
+  </si>
+  <si>
+    <t>pin_responsivity</t>
+  </si>
+  <si>
+    <t>pin_dark_current_na</t>
+  </si>
+  <si>
+    <t>temperature_k</t>
+  </si>
+  <si>
+    <t>rl_ohm</t>
+  </si>
+  <si>
+    <t>tia_gain_ohm</t>
+  </si>
+  <si>
+    <t>tia_noise_pa_rthz</t>
+  </si>
+  <si>
+    <t>host_rx_noise_rms</t>
   </si>
   <si>
     <t>host_tx_noise_rms</t>
   </si>
   <si>
-    <t>module_tx_noise_rms</t>
-  </si>
-  <si>
-    <t>module_rx_noise_rms</t>
-  </si>
-  <si>
-    <t>host_rx_noise_rms</t>
-  </si>
-  <si>
     <t>use_s4p</t>
   </si>
   <si>
@@ -197,13 +218,16 @@
     <t>pol_angle_deg</t>
   </si>
   <si>
-    <t>case_dr_500m_limit</t>
-  </si>
-  <si>
-    <t>case_fr1_2km_limit</t>
-  </si>
-  <si>
-    <t>case_lr1_10km_limit</t>
+    <t>case_cd_dgd_stress</t>
+  </si>
+  <si>
+    <t>case_high_loss</t>
+  </si>
+  <si>
+    <t>case_high_noise</t>
+  </si>
+  <si>
+    <t>case_combined_stress</t>
   </si>
 </sst>
 </file>
@@ -779,7 +803,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -803,7 +827,7 @@
         <v>30</v>
       </c>
       <c r="B3">
-        <v>26.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -819,15 +843,15 @@
         <v>32</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>0.617</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="b">
-        <v>1</v>
+      <c r="B6">
+        <v>-150</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -835,7 +859,7 @@
         <v>34</v>
       </c>
       <c r="B7">
-        <v>0.003</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -843,7 +867,7 @@
         <v>35</v>
       </c>
       <c r="B8">
-        <v>0.003</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -851,7 +875,7 @@
         <v>36</v>
       </c>
       <c r="B9">
-        <v>0.003</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -859,23 +883,23 @@
         <v>37</v>
       </c>
       <c r="B10">
-        <v>0.003</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>38</v>
       </c>
-      <c r="B11" t="b">
-        <v>1</v>
+      <c r="B11">
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
-        <v>48</v>
+      <c r="B12">
+        <v>298.15</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -883,7 +907,7 @@
         <v>40</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -891,7 +915,7 @@
         <v>41</v>
       </c>
       <c r="B14">
-        <v>40000000000</v>
+        <v>720</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -899,7 +923,7 @@
         <v>42</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -907,7 +931,7 @@
         <v>43</v>
       </c>
       <c r="B16">
-        <v>0.25</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -915,30 +939,86 @@
         <v>44</v>
       </c>
       <c r="B17">
-        <v>40000000000</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>45</v>
       </c>
-      <c r="B18">
-        <v>40000000000</v>
+      <c r="B18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>46</v>
       </c>
-      <c r="B19">
-        <v>40000000000</v>
+      <c r="B19" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="b">
+      <c r="B20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26">
+        <v>40000000000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -986,7 +1066,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -994,7 +1074,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B6">
         <v>0.0001</v>
@@ -1002,7 +1082,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B7">
         <v>0.0001</v>
@@ -1010,7 +1090,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B8">
         <v>10000</v>
@@ -1018,7 +1098,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1026,7 +1106,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -1039,27 +1119,39 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="I1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1073,58 +1165,135 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>26.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>-150</v>
+      </c>
+      <c r="F2">
+        <v>25</v>
+      </c>
+      <c r="G2">
+        <v>16</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C3">
-        <v>2.24</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>45</v>
       </c>
       <c r="E3">
-        <v>26.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>-150</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>16</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>-150</v>
+      </c>
+      <c r="F4">
+        <v>25</v>
+      </c>
+      <c r="G4">
+        <v>16</v>
+      </c>
+      <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>-140</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
+        <v>25</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
         <v>45</v>
       </c>
-      <c r="E4">
-        <v>26.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5">
-        <v>28</v>
-      </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5">
-        <v>45</v>
-      </c>
-      <c r="E5">
-        <v>26.5</v>
+      <c r="E6">
+        <v>-142</v>
+      </c>
+      <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>20</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove obsolete baseline optimizers and focus purely on DDPS
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -1101,7 +1101,7 @@
         <v>60</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1109,7 +1109,7 @@
         <v>61</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>